<commit_message>
auto: atualiza paineis -- 15/09/2026 11:32
</commit_message>
<xml_diff>
--- a/Impostos_Retidos_Recolhidos_GDF/resumo_final_impostos_gdf_2026.xlsx
+++ b/Impostos_Retidos_Recolhidos_GDF/resumo_final_impostos_gdf_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Extração Impostos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extração Impostos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Posição 14/09/2026 - 08h</t>
+          <t>Posição 14/09/2026 - 14h</t>
         </is>
       </c>
     </row>
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>82202200.97</v>
+        <v>71965612.45</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>7819500.43</v>
+        <v>64998932.1</v>
       </c>
     </row>
     <row r="7">
@@ -576,10 +576,10 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>2399717.61</v>
+        <v>2370853.79</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>6906.69</v>
+        <v>2353099.41</v>
       </c>
     </row>
     <row r="8">
@@ -599,10 +599,10 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>738846.27</v>
+        <v>447839.71</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>32533.78</v>
+        <v>663272.05</v>
       </c>
     </row>
     <row r="9">
@@ -622,10 +622,10 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>976908.22</v>
+        <v>955152.53</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>53811.99</v>
+        <v>852670.9399999999</v>
       </c>
     </row>
     <row r="10">
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>46128021.61</v>
+        <v>43261006.64</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>4590106.23</v>
+        <v>38859184.89</v>
       </c>
     </row>
     <row r="11">
@@ -668,10 +668,10 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2033442.7</v>
+        <v>1892417.29</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>41871.04</v>
+        <v>1807114.44</v>
       </c>
     </row>
     <row r="12">
@@ -694,7 +694,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1011014.46</v>
+        <v>9717546.65</v>
       </c>
     </row>
     <row r="13">
@@ -717,7 +717,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>12656.28</v>
+        <v>137263.92</v>
       </c>
     </row>
     <row r="14">
@@ -740,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>7881.29</v>
+        <v>2798451.63</v>
       </c>
     </row>
     <row r="15">
@@ -763,7 +763,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>2502.47</v>
+        <v>40661.45</v>
       </c>
     </row>
     <row r="16">
@@ -786,7 +786,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>300.54</v>
+        <v>1576988.27</v>
       </c>
     </row>
     <row r="17">
@@ -809,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>24.51</v>
+        <v>3563.42</v>
       </c>
     </row>
     <row r="18">
@@ -832,7 +832,7 @@
         <v>732.98</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>12279.71</v>
+        <v>24959603.02</v>
       </c>
     </row>
     <row r="19">
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1667303.7</v>
+        <v>1300037.44</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>322955.91</v>
+        <v>874840.1800000001</v>
       </c>
     </row>
     <row r="20">
@@ -875,10 +875,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>83552.42999999999</v>
+        <v>81888.85000000001</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2535.59</v>
+        <v>79050.71000000001</v>
       </c>
     </row>
     <row r="21">
@@ -901,7 +901,7 @@
         <v>472511.11</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>472511.11</v>
+        <v>7674105.49</v>
       </c>
     </row>
     <row r="22">
@@ -924,7 +924,7 @@
         <v>304225.38</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>304225.38</v>
+        <v>5994107.51</v>
       </c>
     </row>
     <row r="23">
@@ -947,7 +947,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>25809.82</v>
+        <v>63895.14</v>
       </c>
     </row>
     <row r="24">
@@ -967,10 +967,10 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>1135881.4</v>
+        <v>979010.24</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>10611818.27</v>
+        <v>116168615.44</v>
       </c>
     </row>
     <row r="25">
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>364488.4</v>
+        <v>339500.55</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>3721921.45</v>
+        <v>34532002.06</v>
       </c>
     </row>
     <row r="26">
@@ -1016,7 +1016,7 @@
         <v>612.25</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>32</v>
+        <v>519.5</v>
       </c>
     </row>
     <row r="27">
@@ -1036,10 +1036,10 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>157514.3</v>
+        <v>131001.86</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>0</v>
+        <v>131001.86</v>
       </c>
     </row>
     <row r="28">
@@ -1059,10 +1059,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>68503.78</v>
+        <v>57456.92</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0</v>
+        <v>57456.92</v>
       </c>
     </row>
     <row r="29">
@@ -1082,10 +1082,10 @@
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>3365329.69</v>
+        <v>3321167.9</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>172956.55</v>
+        <v>3668692.78</v>
       </c>
     </row>
     <row r="30">
@@ -1105,10 +1105,10 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>45220.18</v>
+        <v>41239.4</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>12371.82</v>
+        <v>53611.22</v>
       </c>
     </row>
     <row r="31">
@@ -1131,7 +1131,7 @@
         <v>3084217.71</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>0</v>
+        <v>3538622.77</v>
       </c>
     </row>
     <row r="32">
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="D32" s="6" t="n">
-        <v>14696734.51</v>
+        <v>14254430.63</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>276185.74</v>
+        <v>14188927.83</v>
       </c>
     </row>
     <row r="33">
@@ -1174,10 +1174,10 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>15854932.73</v>
+        <v>15513748.42</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>167584.34</v>
+        <v>15315728.62</v>
       </c>
     </row>
     <row r="34">
@@ -1197,10 +1197,10 @@
         </is>
       </c>
       <c r="D34" s="6" t="n">
+        <v>29852.19</v>
+      </c>
+      <c r="E34" s="6" t="n">
         <v>35591.84</v>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1223,7 +1223,7 @@
         <v>9241.92</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>0</v>
+        <v>9241.92</v>
       </c>
     </row>
     <row r="36">
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>21222.26</v>
+        <v>1742422.36</v>
       </c>
     </row>
     <row r="37">
@@ -1269,7 +1269,7 @@
         <v>0</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>1946.53</v>
+        <v>25074.29</v>
       </c>
     </row>
     <row r="38">
@@ -1292,7 +1292,7 @@
         <v>0</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>375.86</v>
+        <v>294164.57</v>
       </c>
     </row>
     <row r="39">
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>1.98</v>
+        <v>49.08</v>
       </c>
     </row>
     <row r="40">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="D40" s="6" t="n">
-        <v>75974.35000000001</v>
+        <v>66878.75</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>8.720000000000001</v>
+        <v>617836.53</v>
       </c>
     </row>
     <row r="41">
@@ -1358,10 +1358,10 @@
         </is>
       </c>
       <c r="D41" s="8" t="n">
-        <v>67220.61</v>
+        <v>67199.69</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>0</v>
+        <v>67199.69</v>
       </c>
     </row>
     <row r="42">
@@ -1381,10 +1381,10 @@
         </is>
       </c>
       <c r="D42" s="6" t="n">
-        <v>758408.3199999999</v>
+        <v>732585.45</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>17463.62</v>
+        <v>614618.96</v>
       </c>
     </row>
     <row r="43">
@@ -1407,7 +1407,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>341.56</v>
+        <v>532497.2</v>
       </c>
     </row>
     <row r="44">
@@ -1427,10 +1427,10 @@
         </is>
       </c>
       <c r="D44" s="6" t="n">
-        <v>4722435.49</v>
+        <v>3413396.48</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>2348600.74</v>
+        <v>36526970.41</v>
       </c>
     </row>
     <row r="45">
@@ -1450,10 +1450,10 @@
         </is>
       </c>
       <c r="D45" s="8" t="n">
-        <v>4800693.19</v>
+        <v>3486195.58</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>2008431.08</v>
+        <v>28803334.2</v>
       </c>
     </row>
     <row r="46">
@@ -1473,10 +1473,10 @@
         </is>
       </c>
       <c r="D46" s="6" t="n">
-        <v>6028292.17</v>
+        <v>5976391.95</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>297684.78</v>
+        <v>6376475.27</v>
       </c>
     </row>
     <row r="47">
@@ -1496,10 +1496,10 @@
         </is>
       </c>
       <c r="D47" s="8" t="n">
-        <v>742167.84</v>
+        <v>729271.5</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>0</v>
+        <v>782208.54</v>
       </c>
     </row>
     <row r="48">
@@ -1522,7 +1522,7 @@
         <v>0</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>28048.33</v>
+        <v>128888.14</v>
       </c>
     </row>
     <row r="49">
@@ -1542,10 +1542,10 @@
         </is>
       </c>
       <c r="D49" s="8" t="n">
-        <v>3373570.05</v>
+        <v>2776003.74</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>542099.62</v>
+        <v>212291634.78</v>
       </c>
     </row>
     <row r="50">
@@ -1565,10 +1565,10 @@
         </is>
       </c>
       <c r="D50" s="6" t="n">
-        <v>2967333.73</v>
+        <v>2471207.24</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>906648.2</v>
+        <v>11163255</v>
       </c>
     </row>
     <row r="51">
@@ -1588,10 +1588,10 @@
         </is>
       </c>
       <c r="D51" s="8" t="n">
-        <v>268856821.3</v>
+        <v>220543785.96</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>1207681.46</v>
+        <v>219295329.65</v>
       </c>
     </row>
     <row r="52">
@@ -1611,10 +1611,10 @@
         </is>
       </c>
       <c r="D52" s="6" t="n">
-        <v>26964474.89</v>
+        <v>25303821.12</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>1207613.46</v>
+        <v>24058554.7</v>
       </c>
     </row>
     <row r="53">
@@ -1634,10 +1634,10 @@
         </is>
       </c>
       <c r="D53" s="8" t="n">
-        <v>83228662.12</v>
+        <v>70260265.48999999</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>1080958.23</v>
+        <v>132127843.55</v>
       </c>
     </row>
     <row r="54">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="D54" s="6" t="n">
-        <v>23902447.06</v>
+        <v>23606766.96</v>
       </c>
       <c r="E54" s="6" t="n">
         <v>0</v>
@@ -1680,10 +1680,10 @@
         </is>
       </c>
       <c r="D55" s="8" t="n">
-        <v>446887.94</v>
+        <v>365693.2</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>19763.8</v>
+        <v>9399467.869999999</v>
       </c>
     </row>
     <row r="56">
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="D56" s="6" t="n">
-        <v>106308.07</v>
+        <v>103387.69</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>460.11</v>
+        <v>103580.39</v>
       </c>
     </row>
     <row r="57">
@@ -1726,10 +1726,10 @@
         </is>
       </c>
       <c r="D57" s="8" t="n">
-        <v>79762.94</v>
+        <v>77509.96000000001</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>26.65</v>
+        <v>1760934.58</v>
       </c>
     </row>
     <row r="58">
@@ -1749,10 +1749,10 @@
         </is>
       </c>
       <c r="D58" s="6" t="n">
-        <v>8738.5</v>
+        <v>8426.940000000001</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>0</v>
+        <v>8426.940000000001</v>
       </c>
     </row>
     <row r="59">
@@ -1775,7 +1775,7 @@
         <v>257681.12</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>257681.12</v>
+        <v>69818297.03</v>
       </c>
     </row>
     <row r="60">
@@ -1798,7 +1798,7 @@
         <v>204390.58</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>204390.58</v>
+        <v>23218513.1</v>
       </c>
     </row>
     <row r="61">
@@ -1821,7 +1821,7 @@
         <v>0</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>21384.26</v>
+        <v>29734507.26</v>
       </c>
     </row>
     <row r="62">
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>35596.91</v>
+        <v>671457.23</v>
       </c>
     </row>
     <row r="63">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D63" s="8" t="n">
-        <v>1071.3</v>
+        <v>422.4</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>7725.13</v>
+        <v>1237775.49</v>
       </c>
     </row>
     <row r="64">
@@ -1890,7 +1890,7 @@
         <v>0</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>822.34</v>
+        <v>5256.04</v>
       </c>
     </row>
     <row r="65">
@@ -1910,10 +1910,10 @@
         </is>
       </c>
       <c r="D65" s="8" t="n">
-        <v>311403.29</v>
+        <v>287348.23</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>0</v>
+        <v>287148.94</v>
       </c>
     </row>
     <row r="66">
@@ -1936,7 +1936,7 @@
         <v>42733.65</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>0</v>
+        <v>42733.65</v>
       </c>
     </row>
     <row r="67">
@@ -1959,7 +1959,7 @@
         <v>37268.35</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>3377.91</v>
+        <v>14569.41</v>
       </c>
     </row>
     <row r="68">
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>14074.62</v>
+        <v>31327.67</v>
       </c>
     </row>
     <row r="69">
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="D69" s="8" t="n">
-        <v>2070442.41</v>
+        <v>1739230.38</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>291024.91</v>
+        <v>4109873.97</v>
       </c>
     </row>
     <row r="70">
@@ -2025,10 +2025,10 @@
         </is>
       </c>
       <c r="D70" s="6" t="n">
-        <v>2952013.2</v>
+        <v>2521600.37</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>533522.42</v>
+        <v>2820997.83</v>
       </c>
     </row>
     <row r="71">
@@ -2051,7 +2051,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>7250.33</v>
+        <v>356003.68</v>
       </c>
     </row>
     <row r="72">
@@ -2074,7 +2074,7 @@
         <v>2346.02</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>128.78</v>
+        <v>701452.8</v>
       </c>
     </row>
     <row r="73">
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="D73" s="8" t="n">
-        <v>0</v>
+        <v>-2797.31</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>0</v>
+        <v>3754.83</v>
       </c>
     </row>
     <row r="74">
@@ -2117,10 +2117,10 @@
         </is>
       </c>
       <c r="D74" s="6" t="n">
-        <v>211.48</v>
+        <v>105.74</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>134.5</v>
+        <v>973317.26</v>
       </c>
     </row>
     <row r="75">
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>0</v>
+        <v>398.52</v>
       </c>
     </row>
     <row r="76">
@@ -2166,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>44255.5</v>
+        <v>522541.2</v>
       </c>
     </row>
     <row r="77">
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>1393.52</v>
+        <v>25368.29</v>
       </c>
     </row>
     <row r="78">
@@ -2212,7 +2212,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>79490.82000000001</v>
+        <v>476222.92</v>
       </c>
     </row>
     <row r="79">
@@ -2235,7 +2235,7 @@
         <v>0</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>0</v>
+        <v>31992.97</v>
       </c>
     </row>
     <row r="80">
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>0</v>
+        <v>435996.54</v>
       </c>
     </row>
     <row r="81">
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0</v>
+        <v>2470.77</v>
       </c>
     </row>
     <row r="82">
@@ -2304,7 +2304,7 @@
         <v>0</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>217.81</v>
+        <v>230258.76</v>
       </c>
     </row>
     <row r="83">
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84">
@@ -2350,7 +2350,7 @@
         <v>0</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>0</v>
+        <v>392890.91</v>
       </c>
     </row>
     <row r="85">
@@ -2373,7 +2373,7 @@
         <v>0</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>450.55</v>
+        <v>652396.09</v>
       </c>
     </row>
     <row r="86">
@@ -2396,7 +2396,7 @@
         <v>0</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>0</v>
+        <v>138.2</v>
       </c>
     </row>
     <row r="87">
@@ -2419,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>0</v>
+        <v>607085.15</v>
       </c>
     </row>
     <row r="88">
@@ -2442,7 +2442,7 @@
         <v>0</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>0</v>
+        <v>1573.28</v>
       </c>
     </row>
     <row r="89">
@@ -2465,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>0</v>
+        <v>253940.9</v>
       </c>
     </row>
     <row r="90">
@@ -2488,7 +2488,7 @@
         <v>0</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>0</v>
+        <v>914.8</v>
       </c>
     </row>
     <row r="91">
@@ -2511,7 +2511,7 @@
         <v>0</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>58932.13</v>
+        <v>585017.62</v>
       </c>
     </row>
     <row r="92">
@@ -2534,7 +2534,7 @@
         <v>0</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>0</v>
+        <v>75.76000000000001</v>
       </c>
     </row>
     <row r="93">
@@ -2557,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>57750.32</v>
+        <v>534378.58</v>
       </c>
     </row>
     <row r="94">
@@ -2580,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>0</v>
+        <v>32408.84</v>
       </c>
     </row>
     <row r="95">
@@ -2603,7 +2603,7 @@
         <v>0</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>0</v>
+        <v>319207.85</v>
       </c>
     </row>
     <row r="96">
@@ -2626,7 +2626,7 @@
         <v>0</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>0</v>
+        <v>11.26</v>
       </c>
     </row>
     <row r="97">
@@ -2649,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>34990.97</v>
+        <v>260977.61</v>
       </c>
     </row>
     <row r="98">
@@ -2672,7 +2672,7 @@
         <v>0</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>0</v>
+        <v>885.25</v>
       </c>
     </row>
     <row r="99">
@@ -2695,7 +2695,7 @@
         <v>0</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>1585.58</v>
+        <v>348477.13</v>
       </c>
     </row>
     <row r="100">
@@ -2718,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>0</v>
+        <v>30.16</v>
       </c>
     </row>
     <row r="101">
@@ -2741,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>622.77</v>
+        <v>419439.66</v>
       </c>
     </row>
     <row r="102">
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>397.56</v>
+        <v>10507.3</v>
       </c>
     </row>
     <row r="103">
@@ -2787,7 +2787,7 @@
         <v>192.45</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>157.87</v>
+        <v>415950.75</v>
       </c>
     </row>
     <row r="104">
@@ -2810,7 +2810,7 @@
         <v>0</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>68858.7</v>
+        <v>349097.11</v>
       </c>
     </row>
     <row r="105">
@@ -2833,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>0</v>
+        <v>5712.99</v>
       </c>
     </row>
     <row r="106">
@@ -2856,7 +2856,7 @@
         <v>0</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>101.13</v>
+        <v>863123.1899999999</v>
       </c>
     </row>
     <row r="107">
@@ -2879,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>0</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="108">
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>49.53</v>
+        <v>259551.53</v>
       </c>
     </row>
     <row r="109">
@@ -2925,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>71630.48</v>
+        <v>369466.05</v>
       </c>
     </row>
     <row r="110">
@@ -2948,7 +2948,7 @@
         <v>0</v>
       </c>
       <c r="E110" s="6" t="n">
-        <v>0</v>
+        <v>1251.36</v>
       </c>
     </row>
     <row r="111">
@@ -2971,7 +2971,7 @@
         <v>0</v>
       </c>
       <c r="E111" s="8" t="n">
-        <v>0</v>
+        <v>120179</v>
       </c>
     </row>
     <row r="112">
@@ -2994,7 +2994,7 @@
         <v>0</v>
       </c>
       <c r="E112" s="6" t="n">
-        <v>31.25</v>
+        <v>312229.92</v>
       </c>
     </row>
     <row r="113">
@@ -3017,7 +3017,7 @@
         <v>0</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>0</v>
+        <v>191210.9</v>
       </c>
     </row>
     <row r="114">
@@ -3040,7 +3040,7 @@
         <v>0</v>
       </c>
       <c r="E114" s="6" t="n">
-        <v>98.95999999999999</v>
+        <v>219375.8</v>
       </c>
     </row>
     <row r="115">
@@ -3063,7 +3063,7 @@
         <v>0</v>
       </c>
       <c r="E115" s="8" t="n">
-        <v>2677.61</v>
+        <v>509964.14</v>
       </c>
     </row>
     <row r="116">
@@ -3086,7 +3086,7 @@
         <v>0</v>
       </c>
       <c r="E116" s="6" t="n">
-        <v>0</v>
+        <v>164795.22</v>
       </c>
     </row>
     <row r="117">
@@ -3109,7 +3109,7 @@
         <v>0</v>
       </c>
       <c r="E117" s="8" t="n">
-        <v>0</v>
+        <v>1617.69</v>
       </c>
     </row>
     <row r="118">
@@ -3132,7 +3132,7 @@
         <v>0</v>
       </c>
       <c r="E118" s="6" t="n">
-        <v>28087.59</v>
+        <v>252248.78</v>
       </c>
     </row>
     <row r="119">
@@ -3155,7 +3155,7 @@
         <v>0</v>
       </c>
       <c r="E119" s="8" t="n">
-        <v>287.28</v>
+        <v>390494.89</v>
       </c>
     </row>
     <row r="120">
@@ -3178,7 +3178,7 @@
         <v>0</v>
       </c>
       <c r="E120" s="6" t="n">
-        <v>0</v>
+        <v>52.23</v>
       </c>
     </row>
     <row r="121">
@@ -3201,7 +3201,7 @@
         <v>0</v>
       </c>
       <c r="E121" s="8" t="n">
-        <v>0</v>
+        <v>125921.6</v>
       </c>
     </row>
     <row r="122">
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="E122" s="6" t="n">
-        <v>0</v>
+        <v>19231.61</v>
       </c>
     </row>
     <row r="123">
@@ -3247,7 +3247,7 @@
         <v>0</v>
       </c>
       <c r="E123" s="8" t="n">
-        <v>0</v>
+        <v>247422.22</v>
       </c>
     </row>
     <row r="124">
@@ -3270,7 +3270,7 @@
         <v>0</v>
       </c>
       <c r="E124" s="6" t="n">
-        <v>0</v>
+        <v>178.95</v>
       </c>
     </row>
     <row r="125">
@@ -3293,7 +3293,7 @@
         <v>0</v>
       </c>
       <c r="E125" s="8" t="n">
-        <v>86711.60000000001</v>
+        <v>332496.5</v>
       </c>
     </row>
     <row r="126">
@@ -3316,7 +3316,7 @@
         <v>0</v>
       </c>
       <c r="E126" s="6" t="n">
-        <v>0</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="127">
@@ -3339,7 +3339,7 @@
         <v>0</v>
       </c>
       <c r="E127" s="8" t="n">
-        <v>0</v>
+        <v>104548.74</v>
       </c>
     </row>
     <row r="128">
@@ -3362,7 +3362,7 @@
         <v>0</v>
       </c>
       <c r="E128" s="6" t="n">
-        <v>0</v>
+        <v>182.49</v>
       </c>
     </row>
     <row r="129">
@@ -3385,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="E129" s="8" t="n">
-        <v>0</v>
+        <v>195614.75</v>
       </c>
     </row>
     <row r="130">
@@ -3408,7 +3408,7 @@
         <v>0</v>
       </c>
       <c r="E130" s="6" t="n">
-        <v>0</v>
+        <v>61.79</v>
       </c>
     </row>
     <row r="131">
@@ -3431,7 +3431,7 @@
         <v>0</v>
       </c>
       <c r="E131" s="8" t="n">
-        <v>0</v>
+        <v>6430188.16</v>
       </c>
     </row>
     <row r="132">
@@ -3451,10 +3451,10 @@
         </is>
       </c>
       <c r="D132" s="6" t="n">
-        <v>2553800.59</v>
+        <v>2498776.29</v>
       </c>
       <c r="E132" s="6" t="n">
-        <v>1234905.59</v>
+        <v>19799088.38</v>
       </c>
     </row>
     <row r="133">
@@ -3477,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="E133" s="8" t="n">
-        <v>174551.55</v>
+        <v>8893961.369999999</v>
       </c>
     </row>
     <row r="134">
@@ -3500,7 +3500,7 @@
         <v>0</v>
       </c>
       <c r="E134" s="6" t="n">
-        <v>6162.14</v>
+        <v>195995.19</v>
       </c>
     </row>
     <row r="135">
@@ -3520,10 +3520,10 @@
         </is>
       </c>
       <c r="D135" s="8" t="n">
-        <v>956013.5600000001</v>
+        <v>28501.25</v>
       </c>
       <c r="E135" s="8" t="n">
-        <v>13065.73</v>
+        <v>10925979.87</v>
       </c>
     </row>
     <row r="136">
@@ -3543,10 +3543,10 @@
         </is>
       </c>
       <c r="D136" s="6" t="n">
-        <v>2603.46</v>
+        <v>0</v>
       </c>
       <c r="E136" s="6" t="n">
-        <v>14833.98</v>
+        <v>989162.75</v>
       </c>
     </row>
     <row r="137">
@@ -3569,7 +3569,7 @@
         <v>0</v>
       </c>
       <c r="E137" s="8" t="n">
-        <v>0</v>
+        <v>79598.94</v>
       </c>
     </row>
     <row r="138">
@@ -3589,10 +3589,10 @@
         </is>
       </c>
       <c r="D138" s="6" t="n">
-        <v>4109292.23</v>
+        <v>3820769.83</v>
       </c>
       <c r="E138" s="6" t="n">
-        <v>220716.9</v>
+        <v>10819606.75</v>
       </c>
     </row>
     <row r="139">
@@ -3612,10 +3612,10 @@
         </is>
       </c>
       <c r="D139" s="8" t="n">
-        <v>5959270.31</v>
+        <v>5320212.23</v>
       </c>
       <c r="E139" s="8" t="n">
-        <v>28591.56</v>
+        <v>23093010.41</v>
       </c>
     </row>
     <row r="140">
@@ -3635,10 +3635,10 @@
         </is>
       </c>
       <c r="D140" s="6" t="n">
-        <v>5664834.76</v>
+        <v>5200480.33</v>
       </c>
       <c r="E140" s="6" t="n">
-        <v>1886.18</v>
+        <v>5391028.88</v>
       </c>
     </row>
     <row r="141">
@@ -3661,7 +3661,7 @@
         <v>0</v>
       </c>
       <c r="E141" s="8" t="n">
-        <v>0</v>
+        <v>3467281.62</v>
       </c>
     </row>
     <row r="142">
@@ -3681,10 +3681,10 @@
         </is>
       </c>
       <c r="D142" s="6" t="n">
-        <v>5259190.36</v>
+        <v>4840750.16</v>
       </c>
       <c r="E142" s="6" t="n">
-        <v>20444.45</v>
+        <v>4715149.26</v>
       </c>
     </row>
     <row r="143">
@@ -3707,7 +3707,7 @@
         <v>51327.78</v>
       </c>
       <c r="E143" s="8" t="n">
-        <v>81.16</v>
+        <v>6128322.39</v>
       </c>
     </row>
     <row r="144">
@@ -3730,7 +3730,7 @@
         <v>4739.28</v>
       </c>
       <c r="E144" s="6" t="n">
-        <v>0</v>
+        <v>193866.21</v>
       </c>
     </row>
     <row r="145">
@@ -3750,10 +3750,10 @@
         </is>
       </c>
       <c r="D145" s="8" t="n">
-        <v>1192.32</v>
+        <v>0</v>
       </c>
       <c r="E145" s="8" t="n">
-        <v>0</v>
+        <v>2375.3</v>
       </c>
     </row>
     <row r="146">
@@ -3773,10 +3773,10 @@
         </is>
       </c>
       <c r="D146" s="6" t="n">
-        <v>32223.17</v>
+        <v>31715.57</v>
       </c>
       <c r="E146" s="6" t="n">
-        <v>559.27</v>
+        <v>33555.48</v>
       </c>
     </row>
     <row r="147">
@@ -3796,10 +3796,10 @@
         </is>
       </c>
       <c r="D147" s="8" t="n">
-        <v>25751.48</v>
+        <v>5643.98</v>
       </c>
       <c r="E147" s="8" t="n">
-        <v>0</v>
+        <v>5643.98</v>
       </c>
     </row>
     <row r="148">
@@ -3822,7 +3822,7 @@
         <v>3887.55</v>
       </c>
       <c r="E148" s="6" t="n">
-        <v>0</v>
+        <v>3887.55</v>
       </c>
     </row>
     <row r="149">
@@ -3842,10 +3842,10 @@
         </is>
       </c>
       <c r="D149" s="8" t="n">
-        <v>80331.28999999999</v>
+        <v>61634.93</v>
       </c>
       <c r="E149" s="8" t="n">
-        <v>30571.78</v>
+        <v>3993819.36</v>
       </c>
     </row>
     <row r="150">
@@ -3868,7 +3868,7 @@
         <v>27806.29</v>
       </c>
       <c r="E150" s="6" t="n">
-        <v>18211.62</v>
+        <v>332618.84</v>
       </c>
     </row>
     <row r="151">
@@ -3888,10 +3888,10 @@
         </is>
       </c>
       <c r="D151" s="8" t="n">
-        <v>317734.43</v>
+        <v>259440.56</v>
       </c>
       <c r="E151" s="8" t="n">
-        <v>0</v>
+        <v>8775.6</v>
       </c>
     </row>
     <row r="152">
@@ -3911,10 +3911,10 @@
         </is>
       </c>
       <c r="D152" s="6" t="n">
-        <v>79945.19</v>
+        <v>77837.45</v>
       </c>
       <c r="E152" s="6" t="n">
-        <v>0</v>
+        <v>1481.76</v>
       </c>
     </row>
     <row r="153">
@@ -3934,10 +3934,10 @@
         </is>
       </c>
       <c r="D153" s="8" t="n">
-        <v>65217.71</v>
+        <v>23632.26</v>
       </c>
       <c r="E153" s="8" t="n">
-        <v>556234.1800000001</v>
+        <v>3576650.27</v>
       </c>
     </row>
     <row r="154">
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D154" s="6" t="n">
-        <v>37042.69</v>
+        <v>10428.01</v>
       </c>
       <c r="E154" s="6" t="n">
         <v>0</v>
@@ -3983,7 +3983,7 @@
         <v>53106.67</v>
       </c>
       <c r="E155" s="8" t="n">
-        <v>0</v>
+        <v>2810905.46</v>
       </c>
     </row>
     <row r="156">
@@ -4029,7 +4029,7 @@
         <v>0</v>
       </c>
       <c r="E157" s="8" t="n">
-        <v>1303304.43</v>
+        <v>6325646.68</v>
       </c>
     </row>
     <row r="158">
@@ -4052,7 +4052,7 @@
         <v>0</v>
       </c>
       <c r="E158" s="6" t="n">
-        <v>973914.13</v>
+        <v>5797726.56</v>
       </c>
     </row>
     <row r="159">
@@ -4072,10 +4072,10 @@
         </is>
       </c>
       <c r="D159" s="8" t="n">
-        <v>46626687.14</v>
+        <v>44044517.01</v>
       </c>
       <c r="E159" s="8" t="n">
-        <v>162582.21</v>
+        <v>49304467.53</v>
       </c>
     </row>
     <row r="160">
@@ -4095,10 +4095,10 @@
         </is>
       </c>
       <c r="D160" s="6" t="n">
-        <v>6114845.28</v>
+        <v>6045876.69</v>
       </c>
       <c r="E160" s="6" t="n">
-        <v>133190.09</v>
+        <v>5759799.72</v>
       </c>
     </row>
     <row r="161">
@@ -4118,10 +4118,10 @@
         </is>
       </c>
       <c r="D161" s="8" t="n">
-        <v>60123.25</v>
+        <v>54856.2</v>
       </c>
       <c r="E161" s="8" t="n">
-        <v>6053.61</v>
+        <v>205683.82</v>
       </c>
     </row>
     <row r="162">
@@ -4164,10 +4164,10 @@
         </is>
       </c>
       <c r="D163" s="8" t="n">
-        <v>824.1</v>
+        <v>698.55</v>
       </c>
       <c r="E163" s="8" t="n">
-        <v>0</v>
+        <v>698.55</v>
       </c>
     </row>
     <row r="164">
@@ -4190,7 +4190,7 @@
         <v>9207.85</v>
       </c>
       <c r="E164" s="6" t="n">
-        <v>0</v>
+        <v>4799.33</v>
       </c>
     </row>
     <row r="165">
@@ -4233,10 +4233,10 @@
         </is>
       </c>
       <c r="D166" s="6" t="n">
-        <v>69969.12</v>
+        <v>34984.56</v>
       </c>
       <c r="E166" s="6" t="n">
-        <v>0</v>
+        <v>34984.56</v>
       </c>
     </row>
     <row r="167">
@@ -4256,10 +4256,10 @@
         </is>
       </c>
       <c r="D167" s="8" t="n">
-        <v>214841.58</v>
+        <v>15341.58</v>
       </c>
       <c r="E167" s="8" t="n">
-        <v>0</v>
+        <v>15341.58</v>
       </c>
     </row>
     <row r="168">
@@ -4279,10 +4279,10 @@
         </is>
       </c>
       <c r="D168" s="6" t="n">
-        <v>414.9</v>
+        <v>207.45</v>
       </c>
       <c r="E168" s="6" t="n">
-        <v>0</v>
+        <v>207.45</v>
       </c>
     </row>
     <row r="169">
@@ -4302,10 +4302,10 @@
         </is>
       </c>
       <c r="D169" s="8" t="n">
-        <v>243425.49</v>
+        <v>242082.93</v>
       </c>
       <c r="E169" s="8" t="n">
-        <v>0</v>
+        <v>265417.83</v>
       </c>
     </row>
     <row r="170">
@@ -4325,10 +4325,10 @@
         </is>
       </c>
       <c r="D170" s="6" t="n">
-        <v>145377.39</v>
+        <v>145260.79</v>
       </c>
       <c r="E170" s="6" t="n">
-        <v>2357.57</v>
+        <v>170098.32</v>
       </c>
     </row>
     <row r="171">
@@ -4351,7 +4351,7 @@
         <v>0</v>
       </c>
       <c r="E171" s="8" t="n">
-        <v>14892.2</v>
+        <v>7775626.23</v>
       </c>
     </row>
     <row r="172">
@@ -4374,7 +4374,7 @@
         <v>0</v>
       </c>
       <c r="E172" s="6" t="n">
-        <v>6039.57</v>
+        <v>884651.84</v>
       </c>
     </row>
     <row r="173">
@@ -4397,7 +4397,7 @@
         <v>0</v>
       </c>
       <c r="E173" s="8" t="n">
-        <v>48638.19</v>
+        <v>425992.46</v>
       </c>
     </row>
     <row r="174">
@@ -4420,7 +4420,7 @@
         <v>0</v>
       </c>
       <c r="E174" s="6" t="n">
-        <v>1298.56</v>
+        <v>5104.49</v>
       </c>
     </row>
     <row r="175">
@@ -4440,10 +4440,10 @@
         </is>
       </c>
       <c r="D175" s="8" t="n">
-        <v>224011.11</v>
+        <v>216634.96</v>
       </c>
       <c r="E175" s="8" t="n">
-        <v>10045.7</v>
+        <v>216634.96</v>
       </c>
     </row>
     <row r="176">
@@ -4466,7 +4466,7 @@
         <v>75</v>
       </c>
       <c r="E176" s="6" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="177">
@@ -4486,10 +4486,10 @@
         </is>
       </c>
       <c r="D177" s="8" t="n">
-        <v>426819.41</v>
+        <v>379872.28</v>
       </c>
       <c r="E177" s="8" t="n">
-        <v>0</v>
+        <v>444408.58</v>
       </c>
     </row>
     <row r="178">
@@ -4512,7 +4512,7 @@
         <v>3077.16</v>
       </c>
       <c r="E178" s="6" t="n">
-        <v>0</v>
+        <v>3077.16</v>
       </c>
     </row>
     <row r="179">
@@ -4532,7 +4532,7 @@
         </is>
       </c>
       <c r="D179" s="8" t="n">
-        <v>1385.87</v>
+        <v>0</v>
       </c>
       <c r="E179" s="8" t="n">
         <v>0</v>
@@ -4558,7 +4558,7 @@
         <v>0</v>
       </c>
       <c r="E180" s="6" t="n">
-        <v>0</v>
+        <v>73153.03</v>
       </c>
     </row>
     <row r="181">
@@ -4578,10 +4578,10 @@
         </is>
       </c>
       <c r="D181" s="8" t="n">
-        <v>61978.01</v>
+        <v>42779.43</v>
       </c>
       <c r="E181" s="8" t="n">
-        <v>304771.03</v>
+        <v>4880223.14</v>
       </c>
     </row>
     <row r="182">
@@ -4604,7 +4604,7 @@
         <v>0</v>
       </c>
       <c r="E182" s="6" t="n">
-        <v>143327.48</v>
+        <v>1739620.65</v>
       </c>
     </row>
     <row r="183">
@@ -4627,7 +4627,7 @@
         <v>8878.58</v>
       </c>
       <c r="E183" s="8" t="n">
-        <v>0</v>
+        <v>8878.58</v>
       </c>
     </row>
     <row r="184">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="D184" s="6" t="n">
-        <v>250345.38</v>
+        <v>169095.72</v>
       </c>
       <c r="E184" s="6" t="n">
-        <v>0</v>
+        <v>341938.69</v>
       </c>
     </row>
     <row r="185">
@@ -4673,7 +4673,7 @@
         <v>89940.57000000001</v>
       </c>
       <c r="E185" s="8" t="n">
-        <v>0</v>
+        <v>159963.09</v>
       </c>
     </row>
     <row r="186">
@@ -4696,7 +4696,7 @@
         <v>0</v>
       </c>
       <c r="E186" s="6" t="n">
-        <v>500316.82</v>
+        <v>6493361.06</v>
       </c>
     </row>
     <row r="187">
@@ -4719,7 +4719,7 @@
         <v>0</v>
       </c>
       <c r="E187" s="8" t="n">
-        <v>219434.95</v>
+        <v>3631535.14</v>
       </c>
     </row>
     <row r="188">
@@ -4742,7 +4742,7 @@
         <v>0</v>
       </c>
       <c r="E188" s="6" t="n">
-        <v>662238.02</v>
+        <v>5572530</v>
       </c>
     </row>
     <row r="189">
@@ -4765,7 +4765,7 @@
         <v>0</v>
       </c>
       <c r="E189" s="8" t="n">
-        <v>0</v>
+        <v>687.09</v>
       </c>
     </row>
     <row r="190">
@@ -4785,10 +4785,10 @@
         </is>
       </c>
       <c r="D190" s="6" t="n">
-        <v>1299925.32</v>
+        <v>343445.84</v>
       </c>
       <c r="E190" s="6" t="n">
-        <v>5.54</v>
+        <v>13223617.63</v>
       </c>
     </row>
     <row r="191">
@@ -4808,10 +4808,10 @@
         </is>
       </c>
       <c r="D191" s="8" t="n">
-        <v>105074.97</v>
+        <v>92184.98</v>
       </c>
       <c r="E191" s="8" t="n">
-        <v>614.85</v>
+        <v>170698.21</v>
       </c>
     </row>
     <row r="192">
@@ -4834,7 +4834,7 @@
         <v>0</v>
       </c>
       <c r="E192" s="6" t="n">
-        <v>0</v>
+        <v>137559.41</v>
       </c>
     </row>
     <row r="193">
@@ -4854,10 +4854,10 @@
         </is>
       </c>
       <c r="D193" s="8" t="n">
-        <v>520255.84</v>
+        <v>401390.02</v>
       </c>
       <c r="E193" s="8" t="n">
-        <v>45209.76</v>
+        <v>368226.47</v>
       </c>
     </row>
     <row r="194">
@@ -4903,7 +4903,7 @@
         <v>33358</v>
       </c>
       <c r="E195" s="8" t="n">
-        <v>0</v>
+        <v>1815.98</v>
       </c>
     </row>
     <row r="196">
@@ -4926,7 +4926,7 @@
         <v>0</v>
       </c>
       <c r="E196" s="6" t="n">
-        <v>8819.48</v>
+        <v>1656732.63</v>
       </c>
     </row>
     <row r="197">
@@ -4949,7 +4949,7 @@
         <v>0</v>
       </c>
       <c r="E197" s="8" t="n">
-        <v>8444.02</v>
+        <v>469152.28</v>
       </c>
     </row>
     <row r="198">
@@ -4969,10 +4969,10 @@
         </is>
       </c>
       <c r="D198" s="6" t="n">
-        <v>1702653.66</v>
+        <v>1697599.03</v>
       </c>
       <c r="E198" s="6" t="n">
-        <v>8249.540000000001</v>
+        <v>1897092.16</v>
       </c>
     </row>
     <row r="199">
@@ -4992,10 +4992,10 @@
         </is>
       </c>
       <c r="D199" s="8" t="n">
-        <v>18079.25</v>
+        <v>17864.7</v>
       </c>
       <c r="E199" s="8" t="n">
-        <v>24.21</v>
+        <v>17840.49</v>
       </c>
     </row>
     <row r="200">
@@ -5015,10 +5015,10 @@
         </is>
       </c>
       <c r="D200" s="6" t="n">
-        <v>679370237.75</v>
+        <v>679136931.38</v>
       </c>
       <c r="E200" s="6" t="n">
-        <v>86764901.62</v>
+        <v>693830469.65</v>
       </c>
     </row>
     <row r="201">
@@ -5041,7 +5041,7 @@
         <v>0</v>
       </c>
       <c r="E201" s="8" t="n">
-        <v>0</v>
+        <v>257455.8</v>
       </c>
     </row>
     <row r="202">
@@ -5061,10 +5061,10 @@
         </is>
       </c>
       <c r="D202" s="6" t="n">
-        <v>24412.48</v>
+        <v>24387.81</v>
       </c>
       <c r="E202" s="6" t="n">
-        <v>3389.24</v>
+        <v>24191.43</v>
       </c>
     </row>
     <row r="203">
@@ -5084,10 +5084,10 @@
         </is>
       </c>
       <c r="D203" s="8" t="n">
-        <v>417996.43</v>
+        <v>356882.31</v>
       </c>
       <c r="E203" s="8" t="n">
-        <v>10583.5</v>
+        <v>1307788.71</v>
       </c>
     </row>
     <row r="204">
@@ -5107,10 +5107,10 @@
         </is>
       </c>
       <c r="D204" s="6" t="n">
-        <v>908671.36</v>
+        <v>750255.87</v>
       </c>
       <c r="E204" s="6" t="n">
-        <v>36820.92</v>
+        <v>237526.49</v>
       </c>
     </row>
     <row r="205">
@@ -5133,7 +5133,7 @@
         <v>0</v>
       </c>
       <c r="E205" s="8" t="n">
-        <v>4602563.73</v>
+        <v>57447536.32</v>
       </c>
     </row>
     <row r="206">
@@ -5156,7 +5156,7 @@
         <v>0</v>
       </c>
       <c r="E206" s="6" t="n">
-        <v>13765.67</v>
+        <v>790724.42</v>
       </c>
     </row>
     <row r="207">
@@ -5179,7 +5179,7 @@
         <v>392.73</v>
       </c>
       <c r="E207" s="8" t="n">
-        <v>1373.48</v>
+        <v>1415046.96</v>
       </c>
     </row>
     <row r="208">
@@ -5199,10 +5199,10 @@
         </is>
       </c>
       <c r="D208" s="6" t="n">
-        <v>280028.51</v>
+        <v>118156.52</v>
       </c>
       <c r="E208" s="6" t="n">
-        <v>650.05</v>
+        <v>106745.4</v>
       </c>
     </row>
     <row r="209">
@@ -5225,7 +5225,7 @@
         <v>32753.34</v>
       </c>
       <c r="E209" s="8" t="n">
-        <v>0</v>
+        <v>32753.34</v>
       </c>
     </row>
     <row r="210">
@@ -5248,7 +5248,7 @@
         <v>5529.53</v>
       </c>
       <c r="E210" s="6" t="n">
-        <v>2027.87</v>
+        <v>11886187.69</v>
       </c>
     </row>
     <row r="211">
@@ -5271,7 +5271,7 @@
         <v>761.76</v>
       </c>
       <c r="E211" s="8" t="n">
-        <v>61.71</v>
+        <v>3337.28</v>
       </c>
     </row>
     <row r="212">
@@ -5294,7 +5294,7 @@
         <v>0</v>
       </c>
       <c r="E212" s="6" t="n">
-        <v>42267.31</v>
+        <v>31664438.68</v>
       </c>
     </row>
     <row r="213">
@@ -5317,7 +5317,7 @@
         <v>0</v>
       </c>
       <c r="E213" s="8" t="n">
-        <v>30390.17</v>
+        <v>303609.12</v>
       </c>
     </row>
     <row r="214">
@@ -5340,7 +5340,7 @@
         <v>100.97</v>
       </c>
       <c r="E214" s="6" t="n">
-        <v>99131.74000000001</v>
+        <v>4517185.4</v>
       </c>
     </row>
     <row r="215">
@@ -5363,7 +5363,7 @@
         <v>0</v>
       </c>
       <c r="E215" s="8" t="n">
-        <v>7575.48</v>
+        <v>195242.3</v>
       </c>
     </row>
     <row r="216">
@@ -5386,7 +5386,7 @@
         <v>0</v>
       </c>
       <c r="E216" s="6" t="n">
-        <v>104079.08</v>
+        <v>572607.05</v>
       </c>
     </row>
     <row r="217">
@@ -5409,7 +5409,7 @@
         <v>0</v>
       </c>
       <c r="E217" s="8" t="n">
-        <v>545.41</v>
+        <v>6850.71</v>
       </c>
     </row>
     <row r="218">
@@ -5432,7 +5432,7 @@
         <v>95528.72</v>
       </c>
       <c r="E218" s="6" t="n">
-        <v>1327.59</v>
+        <v>25560431.73</v>
       </c>
     </row>
     <row r="219">
@@ -5455,7 +5455,7 @@
         <v>0</v>
       </c>
       <c r="E219" s="8" t="n">
-        <v>0.01</v>
+        <v>1437029.15</v>
       </c>
     </row>
     <row r="220">
@@ -5475,10 +5475,10 @@
         </is>
       </c>
       <c r="D220" s="6" t="n">
-        <v>3691026.6</v>
+        <v>3357783.85</v>
       </c>
       <c r="E220" s="6" t="n">
-        <v>4709.92</v>
+        <v>4105552.21</v>
       </c>
     </row>
     <row r="221">
@@ -5501,7 +5501,7 @@
         <v>0</v>
       </c>
       <c r="E221" s="8" t="n">
-        <v>117309.54</v>
+        <v>42751035.9</v>
       </c>
     </row>
     <row r="222">
@@ -5524,7 +5524,7 @@
         <v>0</v>
       </c>
       <c r="E222" s="6" t="n">
-        <v>23647.66</v>
+        <v>181473.77</v>
       </c>
     </row>
     <row r="223">
@@ -5547,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="E223" s="8" t="n">
-        <v>13309.23</v>
+        <v>597686.8199999999</v>
       </c>
     </row>
     <row r="224">
@@ -5570,7 +5570,7 @@
         <v>0</v>
       </c>
       <c r="E224" s="6" t="n">
-        <v>5111.93</v>
+        <v>137965.67</v>
       </c>
     </row>
     <row r="225">
@@ -5593,7 +5593,7 @@
         <v>0</v>
       </c>
       <c r="E225" s="8" t="n">
-        <v>162911</v>
+        <v>538198.1</v>
       </c>
     </row>
     <row r="226">
@@ -5605,10 +5605,10 @@
       <c r="B226" s="10" t="n"/>
       <c r="C226" s="10" t="n"/>
       <c r="D226" s="11" t="n">
-        <v>1377344869.24</v>
+        <v>1286347312.529999</v>
       </c>
       <c r="E226" s="11" t="n">
-        <v>140220609.64</v>
+        <v>2293785840.950001</v>
       </c>
     </row>
     <row r="229">
@@ -5635,7 +5635,7 @@
         </is>
       </c>
       <c r="B230" s="13" t="n">
-        <v>1385.87</v>
+        <v>0</v>
       </c>
       <c r="C230" s="13" t="n">
         <v>0</v>
@@ -5651,7 +5651,7 @@
         <v>0</v>
       </c>
       <c r="C231" s="13" t="n">
-        <v>53858.15</v>
+        <v>265936.31</v>
       </c>
     </row>
     <row r="232">
@@ -5661,10 +5661,10 @@
         </is>
       </c>
       <c r="B232" s="13" t="n">
-        <v>1266392480.63</v>
+        <v>1182004281.25</v>
       </c>
       <c r="C232" s="13" t="n">
-        <v>128729086.91</v>
+        <v>2080610841.6</v>
       </c>
     </row>
     <row r="233">
@@ -5674,10 +5674,10 @@
         </is>
       </c>
       <c r="B233" s="13" t="n">
-        <v>110951002.74</v>
+        <v>104343031.28</v>
       </c>
       <c r="C233" s="13" t="n">
-        <v>11437664.58</v>
+        <v>212909063.0400001</v>
       </c>
     </row>
     <row r="234">
@@ -5687,10 +5687,10 @@
         </is>
       </c>
       <c r="B234" s="15" t="n">
-        <v>1377344869.24</v>
+        <v>1286347312.529999</v>
       </c>
       <c r="C234" s="15" t="n">
-        <v>140220609.64</v>
+        <v>2293785840.950001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>